<commit_message>
Modelado - Atribución de sentimiento a atributos QUITO ESTANDARIZACIÓN DE SENTIMIENTO. No hace falta.
Actualice los sentimientos de smartband y tv
</commit_message>
<xml_diff>
--- a/data/modelling/atribucion/smartband/df_attr_values_sent.xlsx
+++ b/data/modelling/atribucion/smartband/df_attr_values_sent.xlsx
@@ -425,2061 +425,2427 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>atributo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>n_opi_con_sent</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>sent</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
         <v>10660.5</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>82</v>
       </c>
-      <c r="D2" t="n">
-        <v>1.055855577370933</v>
+      <c r="E2" t="n">
+        <v>0.6867183994325432</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
         <v>5012.5</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>120</v>
       </c>
-      <c r="D3" t="n">
-        <v>0.2631702585882758</v>
+      <c r="E3" t="n">
+        <v>0.5899300851949941</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
         <v>3385</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>79</v>
       </c>
-      <c r="D4" t="n">
-        <v>-0.6234949305327382</v>
+      <c r="E4" t="n">
+        <v>0.4816666584420749</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="n">
         <v>6444.5</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>103</v>
       </c>
-      <c r="D5" t="n">
-        <v>0.884319034583219</v>
+      <c r="E5" t="n">
+        <v>0.6657734766325888</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="n">
         <v>17689.5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>60</v>
       </c>
-      <c r="D6" t="n">
-        <v>-1.868746293813093</v>
+      <c r="E6" t="n">
+        <v>0.3296192098542681</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="n">
         <v>1495</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>128</v>
       </c>
-      <c r="D7" t="n">
-        <v>-0.09134947909007532</v>
+      <c r="E7" t="n">
+        <v>0.546642582625221</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="n">
         <v>7930</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>85</v>
       </c>
-      <c r="D8" t="n">
-        <v>0.3802458328934776</v>
+      <c r="E8" t="n">
+        <v>0.6042252250277786</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Xiaomi</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>102</v>
       </c>
-      <c r="D9" t="n">
-        <v>0.899121363459184</v>
+      <c r="E9" t="n">
+        <v>0.6328875445807295</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Imilab</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>43</v>
       </c>
-      <c r="D10" t="n">
-        <v>1.211422833854932</v>
+      <c r="E10" t="n">
+        <v>0.6975344995007392</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Samsung</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>10</v>
       </c>
-      <c r="D11" t="n">
-        <v>-2.013367531221349</v>
+      <c r="E11" t="n">
+        <v>0.02999720903140109</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Microwear</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
         <v>31</v>
       </c>
-      <c r="D12" t="n">
-        <v>-0.1939978385867257</v>
+      <c r="E12" t="n">
+        <v>0.4066099427259898</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Amazfit</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
         <v>92</v>
       </c>
-      <c r="D13" t="n">
-        <v>0.8929748307109314</v>
+      <c r="E13" t="n">
+        <v>0.6316152014662795</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Smart Bracelet D20</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>10</v>
       </c>
-      <c r="D14" t="n">
-        <v>-0.9875483880610821</v>
+      <c r="E14" t="n">
+        <v>0.2423435800553</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Haylou</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
         <v>30</v>
       </c>
-      <c r="D15" t="n">
-        <v>1.040277639773483</v>
+      <c r="E15" t="n">
+        <v>0.6621071426184951</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>DT NO.1</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
         <v>28</v>
       </c>
-      <c r="D16" t="n">
-        <v>0.7049543608315747</v>
+      <c r="E16" t="n">
+        <v>0.5926946327448864</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Colmi</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
         <v>21</v>
       </c>
-      <c r="D17" t="n">
-        <v>0.9450687180310372</v>
+      <c r="E17" t="n">
+        <v>0.6423987279764921</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Nictom</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>51</v>
       </c>
-      <c r="D18" t="n">
-        <v>0.7317908370472577</v>
+      <c r="E18" t="n">
+        <v>0.5982498306308545</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Mia</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
         <v>20</v>
       </c>
-      <c r="D19" t="n">
-        <v>0.9317145594387042</v>
+      <c r="E19" t="n">
+        <v>0.6396343936061825</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Huawei</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
         <v>11</v>
       </c>
-      <c r="D20" t="n">
-        <v>0.1119379998726587</v>
+      <c r="E20" t="n">
+        <v>0.4699392006133662</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>You</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
         <v>31</v>
       </c>
-      <c r="D21" t="n">
-        <v>0.7289180156124762</v>
+      <c r="E21" t="n">
+        <v>0.5976551515294329</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>Kospet</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>2</v>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>BlueStar</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>Genérica</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
         <v>12</v>
       </c>
-      <c r="D24" t="n">
-        <v>-0.467577057749842</v>
+      <c r="E24" t="n">
+        <v>0.3499785620735783</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>Shirajo</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
         <v>14</v>
       </c>
-      <c r="D25" t="n">
-        <v>0.1181342791259239</v>
+      <c r="E25" t="n">
+        <v>0.4712218413420506</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>Belmotec</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
         <v>3</v>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>Kingwear</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
         <v>49</v>
       </c>
-      <c r="D27" t="n">
-        <v>1.191426755195605</v>
+      <c r="E27" t="n">
+        <v>0.6933952759676946</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>SmartWatches</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
         <v>29</v>
       </c>
-      <c r="D28" t="n">
-        <v>0.3698076789587996</v>
+      <c r="E28" t="n">
+        <v>0.5233186787759067</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>PSP_BAND</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
         <v>8</v>
       </c>
-      <c r="D29" t="n">
-        <v>-1.027783232399406</v>
+      <c r="E29" t="n">
+        <v>0.2340148963483128</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>Gadnic</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
         <v>1</v>
       </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>Goufit</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
         <v>3</v>
       </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>Netmak</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
         <v>16</v>
       </c>
-      <c r="D32" t="n">
-        <v>0.05049564068011295</v>
+      <c r="E32" t="n">
+        <v>0.457220523945382</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>Honor</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
         <v>10</v>
       </c>
-      <c r="D33" t="n">
-        <v>-0.276023949561949</v>
+      <c r="E33" t="n">
+        <v>0.389630393152434</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>Motorola</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
         <v>1</v>
       </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="B35" t="inlineStr">
         <is>
           <t>Noga</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
         <v>19</v>
       </c>
-      <c r="D35" t="n">
-        <v>-0.3089983889080233</v>
+      <c r="E35" t="n">
+        <v>0.3828046260780203</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" t="inlineStr">
         <is>
           <t>Daikon</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
         <v>3</v>
       </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>Mibro</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
         <v>2</v>
       </c>
-      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>Daza</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>HiFuture</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B40" t="inlineStr">
         <is>
           <t>Ruffo</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
         <v>1</v>
       </c>
-      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>HDT8</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
         <v>4</v>
       </c>
-      <c r="D41" t="n">
-        <v>-1.928617288657353</v>
+      <c r="E41" t="n">
+        <v>0.04754065864613308</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>OEM</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
         <v>8</v>
       </c>
-      <c r="D42" t="n">
-        <v>-1.231489629931741</v>
+      <c r="E42" t="n">
+        <v>0.1918473129504419</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>Doogee</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>Level Up</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>Rohs</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="B46" t="inlineStr">
         <is>
           <t>ISANFIT</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B47" t="inlineStr">
         <is>
           <t>Veryfit</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
         <v>4</v>
       </c>
-      <c r="D47" t="n">
-        <v>-1.70273178450078</v>
+      <c r="E47" t="n">
+        <v>0.09429935621418792</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B48" t="inlineStr">
         <is>
           <t>Phull</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>Haxly</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>M5</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B51" t="inlineStr">
         <is>
           <t>Soul</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B52" t="inlineStr">
         <is>
           <t>Integra</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
         <v>17</v>
       </c>
-      <c r="D52" t="n">
-        <v>0.8998556324164519</v>
+      <c r="E52" t="n">
+        <v>0.6330395395493075</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B53" t="inlineStr">
         <is>
           <t>Mistral</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="B54" t="inlineStr">
         <is>
           <t>Uprint</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>WICKPRO</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="B56" t="inlineStr">
         <is>
           <t>ONCELULAR2</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B57" t="inlineStr">
         <is>
           <t>T-Go</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
         <v>8</v>
       </c>
-      <c r="D57" t="n">
-        <v>-0.6897660554308787</v>
+      <c r="E57" t="n">
+        <v>0.303985047862434</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B58" t="inlineStr">
         <is>
           <t>IWO</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B59" t="inlineStr">
         <is>
           <t>JAZAK</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
         <v>1</v>
       </c>
-      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B60" t="inlineStr">
         <is>
           <t>LCS</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
         <v>1</v>
       </c>
-      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B61" t="inlineStr">
         <is>
           <t>Tressa</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>0</v>
-      </c>
-      <c r="D61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="B62" t="inlineStr">
         <is>
           <t>WickPro</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="B63" t="inlineStr">
         <is>
           <t>Stone</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>Suono</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B65" t="inlineStr">
         <is>
           <t>SLA</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>0</v>
-      </c>
-      <c r="D65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B66" t="inlineStr">
         <is>
           <t>Kanji</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>0</v>
-      </c>
-      <c r="D66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>Solana</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>0</v>
-      </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B68" t="inlineStr">
         <is>
           <t>X8</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B69" t="inlineStr">
         <is>
           <t>LEZAYA</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="B70" t="inlineStr">
         <is>
           <t>Reloj Smartband M6</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" t="inlineStr"/>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B71" t="inlineStr">
         <is>
           <t>SMART WATCH BRACELET</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Marca</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
-        <v>0</v>
-      </c>
-      <c r="D71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" t="n">
+      <c r="A72" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B72" t="n">
         <v>185</v>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>Capacidad de la batería</t>
         </is>
       </c>
-      <c r="C72" t="n">
+      <c r="D72" t="n">
         <v>119</v>
       </c>
-      <c r="D72" t="n">
-        <v>0.5128526212504075</v>
+      <c r="E72" t="n">
+        <v>0.156878134931199</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="n">
+      <c r="A73" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B73" t="n">
         <v>142</v>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Capacidad de la batería</t>
         </is>
       </c>
-      <c r="C73" t="n">
+      <c r="D73" t="n">
         <v>70</v>
       </c>
-      <c r="D73" t="n">
-        <v>-0.04779369282183864</v>
+      <c r="E73" t="n">
+        <v>0.0966122301475693</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="n">
+      <c r="A74" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B74" t="n">
         <v>375</v>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>Capacidad de la batería</t>
         </is>
       </c>
-      <c r="C74" t="n">
+      <c r="D74" t="n">
         <v>95</v>
       </c>
-      <c r="D74" t="n">
-        <v>0.7393994135284503</v>
+      <c r="E74" t="n">
+        <v>0.1812304709223099</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="n">
+      <c r="A75" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B75" t="n">
         <v>296</v>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Capacidad de la batería</t>
         </is>
       </c>
-      <c r="C75" t="n">
+      <c r="D75" t="n">
         <v>61</v>
       </c>
-      <c r="D75" t="n">
-        <v>-0.2738141743229234</v>
+      <c r="E75" t="n">
+        <v>0.07231646920988263</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="n">
+      <c r="A76" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B76" t="n">
         <v>240</v>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>Capacidad de la batería</t>
         </is>
       </c>
-      <c r="C76" t="n">
+      <c r="D76" t="n">
         <v>102</v>
       </c>
-      <c r="D76" t="n">
-        <v>0.8911370887423397</v>
+      <c r="E76" t="n">
+        <v>0.1975413037183161</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="n">
+      <c r="A77" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B77" t="n">
         <v>82.5</v>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>Capacidad de la batería</t>
         </is>
       </c>
-      <c r="C77" t="n">
+      <c r="D77" t="n">
         <v>39</v>
       </c>
-      <c r="D77" t="n">
-        <v>-1.821781256376436</v>
+      <c r="E77" t="n">
+        <v>-0.09408012421034714</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="n">
+      <c r="A78" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B78" t="n">
         <v>168</v>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>Duración de la batería</t>
         </is>
       </c>
-      <c r="C78" t="n">
+      <c r="D78" t="n">
         <v>91</v>
       </c>
-      <c r="D78" t="n">
-        <v>0.5595477917045737</v>
+      <c r="E78" t="n">
+        <v>0.2348293408662897</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="n">
+      <c r="A79" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B79" t="n">
         <v>288</v>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>Duración de la batería</t>
         </is>
       </c>
-      <c r="C79" t="n">
+      <c r="D79" t="n">
         <v>111</v>
       </c>
-      <c r="D79" t="n">
-        <v>0.2719995332055359</v>
+      <c r="E79" t="n">
+        <v>0.199780556655212</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="n">
+      <c r="A80" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B80" t="n">
         <v>468</v>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>Duración de la batería</t>
         </is>
       </c>
-      <c r="C80" t="n">
+      <c r="D80" t="n">
         <v>115</v>
       </c>
-      <c r="D80" t="n">
-        <v>0.6489298281825794</v>
+      <c r="E80" t="n">
+        <v>0.2457239702589931</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="n">
+      <c r="A81" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B81" t="n">
         <v>56</v>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>Duración de la batería</t>
         </is>
       </c>
-      <c r="C81" t="n">
+      <c r="D81" t="n">
         <v>25</v>
       </c>
-      <c r="D81" t="n">
-        <v>-1.480477153092689</v>
+      <c r="E81" t="n">
+        <v>-0.01382594381057517</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="n">
+      <c r="A82" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B82" t="n">
         <v>40.64</v>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>Tamaño de la pantalla</t>
         </is>
       </c>
-      <c r="C82" t="n">
+      <c r="D82" t="n">
         <v>66</v>
       </c>
-      <c r="D82" t="n">
-        <v>0.8238185741505839</v>
+      <c r="E82" t="n">
+        <v>0.4255919605180238</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="n">
+      <c r="A83" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B83" t="n">
         <v>30.099</v>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>Tamaño de la pantalla</t>
         </is>
       </c>
-      <c r="C83" t="n">
+      <c r="D83" t="n">
         <v>89</v>
       </c>
-      <c r="D83" t="n">
-        <v>0.4358885755785805</v>
+      <c r="E83" t="n">
+        <v>0.3562763701769225</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="n">
+      <c r="A84" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B84" t="n">
         <v>43.22499999999999</v>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>Tamaño de la pantalla</t>
         </is>
       </c>
-      <c r="C84" t="n">
+      <c r="D84" t="n">
         <v>16</v>
       </c>
-      <c r="D84" t="n">
-        <v>-0.6770457472582471</v>
+      <c r="E84" t="n">
+        <v>0.1574165246319025</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="n">
+      <c r="A85" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B85" t="n">
         <v>34.163</v>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>Tamaño de la pantalla</t>
         </is>
       </c>
-      <c r="C85" t="n">
+      <c r="D85" t="n">
         <v>55</v>
       </c>
-      <c r="D85" t="n">
-        <v>-0.484824784060277</v>
+      <c r="E85" t="n">
+        <v>0.191762694273458</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="n">
+      <c r="A86" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B86" t="n">
         <v>37.33799999999999</v>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>Tamaño de la pantalla</t>
         </is>
       </c>
-      <c r="C86" t="n">
+      <c r="D86" t="n">
         <v>50</v>
       </c>
-      <c r="D86" t="n">
-        <v>1.261251925820264</v>
+      <c r="E86" t="n">
+        <v>0.5037528429387796</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
+      <c r="A87" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B87" t="n">
         <v>19.335</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>Tamaño de la pantalla</t>
         </is>
       </c>
-      <c r="C87" t="n">
+      <c r="D87" t="n">
         <v>13</v>
       </c>
-      <c r="D87" t="n">
-        <v>-1.359088544230904</v>
+      <c r="E87" t="n">
+        <v>0.03554866371863861</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="n">
+      <c r="A88" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B88" t="n">
         <v>52.479</v>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Tamaño de la pantalla</t>
         </is>
       </c>
-      <c r="C88" t="n">
+      <c r="D88" t="n">
         <v>2</v>
       </c>
-      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B89" t="inlineStr">
         <is>
           <t>AMOLED</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C89" t="n">
+      <c r="D89" t="n">
         <v>123</v>
       </c>
-      <c r="D89" t="n">
-        <v>0.8989412771858279</v>
+      <c r="E89" t="n">
+        <v>0.4780949458436305</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B90" t="inlineStr">
         <is>
           <t>LCD TFT</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C90" t="n">
+      <c r="D90" t="n">
         <v>76</v>
       </c>
-      <c r="D90" t="n">
-        <v>0.8175982199607241</v>
+      <c r="E90" t="n">
+        <v>0.4614161403084724</v>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B91" t="inlineStr">
         <is>
           <t>LCD IPS</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C91" t="n">
+      <c r="D91" t="n">
         <v>19</v>
       </c>
-      <c r="D91" t="n">
-        <v>-0.6998655058010271</v>
+      <c r="E91" t="n">
+        <v>0.1502711790538601</v>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B92" t="inlineStr">
         <is>
           <t>LTPS</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C92" t="n">
+      <c r="D92" t="n">
         <v>2</v>
       </c>
-      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B93" t="inlineStr">
         <is>
           <t>SAMOLED</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C93" t="n">
+      <c r="D93" t="n">
         <v>9</v>
       </c>
-      <c r="D93" t="n">
-        <v>-1.016673991345525</v>
+      <c r="E93" t="n">
+        <v>0.08531189054738048</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B94" t="inlineStr">
         <is>
           <t>Táctil</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C94" t="n">
-        <v>0</v>
-      </c>
-      <c r="D94" t="inlineStr"/>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B95" t="inlineStr">
         <is>
           <t>IPS</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C95" t="n">
+      <c r="D95" t="n">
         <v>6</v>
       </c>
-      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B96" t="inlineStr">
         <is>
           <t>LCD</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C96" t="n">
+      <c r="D96" t="n">
         <v>5</v>
       </c>
-      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B97" t="inlineStr">
         <is>
           <t>OLED</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C97" t="n">
-        <v>0</v>
-      </c>
-      <c r="D97" t="inlineStr"/>
+      <c r="D97" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B98" t="inlineStr">
         <is>
           <t>TFT</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>Tipo de pantalla</t>
         </is>
       </c>
-      <c r="C98" t="n">
+      <c r="D98" t="n">
         <v>4</v>
       </c>
-      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B99" t="inlineStr">
         <is>
           <t>Silicona</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C99" t="n">
+      <c r="D99" t="n">
         <v>244</v>
       </c>
-      <c r="D99" t="n">
-        <v>1.234950459141323</v>
+      <c r="E99" t="n">
+        <v>0.463394323703906</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B100" t="inlineStr">
         <is>
           <t>TPU/Aleación de aluminio</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C100" t="n">
+      <c r="D100" t="n">
         <v>11</v>
       </c>
-      <c r="D100" t="n">
-        <v>-0.1232981474784827</v>
+      <c r="E100" t="n">
+        <v>0.1821612299426851</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B101" t="inlineStr">
         <is>
           <t>Elastómero termoplástico/Aleación de aluminio</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C101" t="n">
+      <c r="D101" t="n">
         <v>11</v>
       </c>
-      <c r="D101" t="n">
-        <v>-0.6520726408526637</v>
+      <c r="E101" t="n">
+        <v>0.07267546573952768</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
+      <c r="A102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B102" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C102" t="n">
+      <c r="D102" t="n">
         <v>36</v>
       </c>
-      <c r="D102" t="n">
-        <v>0.001251172932257644</v>
+      <c r="E102" t="n">
+        <v>0.2079498746239712</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="A103" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B103" t="inlineStr">
         <is>
           <t>Caucho de silicona</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C103" t="n">
+      <c r="D103" t="n">
         <v>17</v>
       </c>
-      <c r="D103" t="n">
-        <v>-0.3060680595009452</v>
+      <c r="E103" t="n">
+        <v>0.1443176808648312</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
+      <c r="A104" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B104" t="inlineStr">
         <is>
           <t>Fluoroelastómero</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C104" t="n">
+      <c r="D104" t="n">
         <v>17</v>
       </c>
-      <c r="D104" t="n">
-        <v>0.4858723588604913</v>
+      <c r="E104" t="n">
+        <v>0.3082934455700955</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
+      <c r="A105" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B105" t="inlineStr">
         <is>
           <t>Cuero</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C105" t="n">
+      <c r="D105" t="n">
         <v>11</v>
       </c>
-      <c r="D105" t="n">
-        <v>-0.1500954042005175</v>
+      <c r="E105" t="n">
+        <v>0.1766127056331284</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
+      <c r="A106" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B106" t="inlineStr">
         <is>
           <t>Acero inoxidable</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C106" t="n">
+      <c r="D106" t="n">
         <v>35</v>
       </c>
-      <c r="D106" t="n">
-        <v>2.266885902735144</v>
+      <c r="E106" t="n">
+        <v>0.6770624224225845</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
+      <c r="A107" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B107" t="inlineStr">
         <is>
           <t>Caucho</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C107" t="n">
-        <v>0</v>
-      </c>
-      <c r="D107" t="inlineStr"/>
+      <c r="D107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
+      <c r="A108" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B108" t="inlineStr">
         <is>
           <t>Plástico</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="C108" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C108" t="n">
+      <c r="D108" t="n">
         <v>13</v>
       </c>
-      <c r="D108" t="n">
-        <v>-0.8510639781586837</v>
+      <c r="E108" t="n">
+        <v>0.03147317836039584</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
+      <c r="A109" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B109" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C109" t="n">
-        <v>0</v>
-      </c>
-      <c r="D109" t="inlineStr"/>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
+      <c r="A110" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B110" t="inlineStr">
         <is>
           <t>Acero inoxidable/Silicona</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C110" t="n">
+      <c r="D110" t="n">
         <v>6</v>
       </c>
-      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
+      <c r="A111" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B111" t="inlineStr">
         <is>
           <t>1ra Cuero/TPU - 2da Silicona negra</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C111" t="n">
-        <v>0</v>
-      </c>
-      <c r="D111" t="inlineStr"/>
+      <c r="D111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
+      <c r="A112" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B112" t="inlineStr">
         <is>
           <t>1ra Metal - 2da Silicona</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C112" t="n">
-        <v>0</v>
-      </c>
-      <c r="D112" t="inlineStr"/>
+      <c r="D112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
+      <c r="A113" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B113" t="inlineStr">
         <is>
           <t>Cuero Genuino</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="C113" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C113" t="n">
+      <c r="D113" t="n">
         <v>7</v>
       </c>
-      <c r="D113" t="n">
-        <v>-0.9850195854167664</v>
+      <c r="E113" t="n">
+        <v>0.003736908525665338</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
+      <c r="A114" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B114" t="inlineStr">
         <is>
           <t>Rosa / negra</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="C114" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C114" t="n">
+      <c r="D114" t="n">
         <v>7</v>
       </c>
-      <c r="D114" t="n">
-        <v>-0.9213420780611582</v>
+      <c r="E114" t="n">
+        <v>0.01692169834200662</v>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
+      <c r="A115" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B115" t="inlineStr">
         <is>
           <t>Resina</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="C115" t="inlineStr">
         <is>
           <t>Material de la malla</t>
         </is>
       </c>
-      <c r="C115" t="n">
-        <v>0</v>
-      </c>
-      <c r="D115" t="inlineStr"/>
+      <c r="D115" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" t="n">
+      <c r="A116" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B116" t="n">
         <v>1</v>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>Es resistente al agua</t>
         </is>
       </c>
-      <c r="C116" t="n">
+      <c r="D116" t="n">
         <v>391</v>
       </c>
-      <c r="D116" t="n">
-        <v>0.7071067811865475</v>
+      <c r="E116" t="n">
+        <v>0.4661149878034115</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="n">
-        <v>0</v>
-      </c>
-      <c r="B117" t="inlineStr">
+      <c r="A117" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B117" t="n">
+        <v>0</v>
+      </c>
+      <c r="C117" t="inlineStr">
         <is>
           <t>Es resistente al agua</t>
         </is>
       </c>
-      <c r="C117" t="n">
+      <c r="D117" t="n">
         <v>55</v>
       </c>
-      <c r="D117" t="n">
-        <v>-0.7071067811865475</v>
+      <c r="E117" t="n">
+        <v>0.2968168254415011</v>
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="n">
+      <c r="A118" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B118" t="n">
         <v>0.0126</v>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="C118" t="n">
+      <c r="D118" t="n">
         <v>60</v>
       </c>
-      <c r="D118" t="n">
-        <v>0.1925106771872289</v>
+      <c r="E118" t="n">
+        <v>0.4578263312070821</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="n">
+      <c r="A119" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B119" t="n">
         <v>0.054</v>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="C119" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="C119" t="n">
+      <c r="D119" t="n">
         <v>58</v>
       </c>
-      <c r="D119" t="n">
-        <v>-0.6218721972333383</v>
+      <c r="E119" t="n">
+        <v>0.425148634731482</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="n">
+      <c r="A120" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B120" t="n">
         <v>0.0384</v>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="C120" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="C120" t="n">
+      <c r="D120" t="n">
         <v>68</v>
       </c>
-      <c r="D120" t="n">
-        <v>-0.8997785151478557</v>
+      <c r="E120" t="n">
+        <v>0.4139974445595084</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="n">
+      <c r="A121" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B121" t="n">
         <v>0.0247</v>
       </c>
-      <c r="B121" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>
       </c>
-      <c r="C121" t="n">
+      <c r="D121" t="n">
         <v>61</v>
       </c>
-      <c r="D121" t="n">
-        <v>1.329140035193965</v>
+      <c r="E121" t="n">
+        <v>0.5034343987792632</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="n">
-        <v>0</v>
-      </c>
-      <c r="B122" t="inlineStr">
+      <c r="A122" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B122" t="n">
+        <v>0</v>
+      </c>
+      <c r="C122" t="inlineStr">
         <is>
           <t>Con pantalla táctil</t>
         </is>
       </c>
-      <c r="C122" t="n">
+      <c r="D122" t="n">
         <v>57</v>
       </c>
-      <c r="D122" t="n">
-        <v>-0.7071067811865474</v>
+      <c r="E122" t="n">
+        <v>0.2312934490571912</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="n">
+      <c r="A123" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B123" t="n">
+        <v>1</v>
+      </c>
+      <c r="C123" t="inlineStr">
         <is>
           <t>Con pantalla táctil</t>
         </is>
       </c>
-      <c r="C123" t="n">
+      <c r="D123" t="n">
         <v>258</v>
       </c>
-      <c r="D123" t="n">
-        <v>0.7071067811865478</v>
+      <c r="E123" t="n">
+        <v>0.3348798819290331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>